<commit_message>
2023-05-18  Oms bug 修复
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/CustomerExport.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/CustomerExport.xlsx
@@ -14,18 +14,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
-  <si>
-    <t>单据类型</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>{.code}</t>
   </si>
   <si>
-    <t>客户单号</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>{.name}</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -34,55 +27,71 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>启用状态</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.disabledName}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>使用组织</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.useOrgName}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>客户分组</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.groupName}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>最新审核人</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.approveUserName}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.createUserName}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>创建人</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>创建时间</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.createTime}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>客户编码</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>简称</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>{.shortName}</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>启用状态</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.disabledName}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用组织</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.useOrgName}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>客户分组</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.groupName}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>最新审核人</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.approveUserName}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.createUserName}</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>创建人</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>创建时间</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{.createTime}</t>
+    <t>单据状态</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.approveStatusName}</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -431,78 +440,85 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="23.625" customWidth="1"/>
-    <col min="2" max="2" width="25.625" customWidth="1"/>
-    <col min="3" max="3" width="20.625" customWidth="1"/>
-    <col min="4" max="4" width="22.375" customWidth="1"/>
-    <col min="5" max="5" width="20.625" customWidth="1"/>
-    <col min="6" max="6" width="20.125" customWidth="1"/>
-    <col min="7" max="9" width="20.625" customWidth="1"/>
+    <col min="2" max="2" width="35.625" customWidth="1"/>
+    <col min="3" max="3" width="38.25" customWidth="1"/>
+    <col min="4" max="4" width="20.625" customWidth="1"/>
+    <col min="5" max="5" width="22.375" customWidth="1"/>
+    <col min="6" max="6" width="20.625" customWidth="1"/>
+    <col min="7" max="7" width="20.125" customWidth="1"/>
+    <col min="8" max="10" width="20.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>16</v>
+      <c r="I2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
-      <c r="C3" s="2"/>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="D3" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>